<commit_message>
Actualiza la demo 2026-10-08 13:34
</commit_message>
<xml_diff>
--- a/docs/ejemplos/evaluacion-prt-ejemplo-FICTICIA.xlsx
+++ b/docs/ejemplos/evaluacion-prt-ejemplo-FICTICIA.xlsx
@@ -551,7 +551,7 @@
         <v>20</v>
       </c>
       <c r="C5" t="str">
-        <v>Piso del puntaje diario (0 a 99); 0 = sin piso</v>
+        <v>% base: mínimo garantizado del puntaje diario (0 a 99); 0 = sin base</v>
       </c>
     </row>
   </sheetData>
@@ -632,7 +632,7 @@
         <v>1</v>
       </c>
       <c r="H2">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="I2" t="str">
         <v>SI</v>
@@ -664,7 +664,7 @@
         <v>1</v>
       </c>
       <c r="H3">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="I3" t="str">
         <v>SI</v>
@@ -696,7 +696,7 @@
         <v>1</v>
       </c>
       <c r="H4">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="I4" t="str">
         <v>SI</v>
@@ -728,7 +728,7 @@
         <v>1</v>
       </c>
       <c r="H5">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="I5" t="str">
         <v>SI</v>
@@ -760,7 +760,7 @@
         <v>1</v>
       </c>
       <c r="H6">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="I6" t="str">
         <v>SI</v>
@@ -792,7 +792,7 @@
         <v>1</v>
       </c>
       <c r="H7">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="I7" t="str">
         <v>SI</v>
@@ -824,7 +824,7 @@
         <v>1</v>
       </c>
       <c r="H8">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="I8" t="str">
         <v>SI</v>
@@ -856,7 +856,7 @@
         <v>1</v>
       </c>
       <c r="H9">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="I9" t="str">
         <v>SI</v>
@@ -888,7 +888,7 @@
         <v>1</v>
       </c>
       <c r="H10">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="I10" t="str">
         <v>SI</v>

</xml_diff>